<commit_message>
feat: implement Excel-to-XML generation in C# and XML parsing in C++
</commit_message>
<xml_diff>
--- a/data/input/RailwaySignals.xlsx
+++ b/data/input/RailwaySignals.xlsx
@@ -1,31 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Debian\home\debian\repo\Railway-Signaling-Data-Generator\data\input\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83360993-88F2-4C8A-A774-DA6FB5FCCC22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Feuil1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
   <si>
     <t>SignalID</t>
   </si>
@@ -88,27 +77,36 @@
   </si>
   <si>
     <t>TRACK03</t>
+  </si>
+  <si>
+    <t>SIG005</t>
+  </si>
+  <si>
+    <t>direct</t>
+  </si>
+  <si>
+    <t>red</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -418,11 +416,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" defaultColWidth="8.88671875" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -442,7 +440,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" ht="28.8" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -462,7 +460,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" ht="28.8" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -482,7 +480,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -502,7 +500,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" ht="28.8" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -520,6 +518,26 @@
       </c>
       <c r="F5" s="2" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6">
+        <v>2000</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>